<commit_message>
fix: META_UNIDAD como desplegable con unidades oficiales MDeIA
Las encuestas estudiantil, docente y administración usan lista fija del catálogo unidades_academicas.json en Google Forms y plantillas Excel.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/plantillas/encuestas/plantilla-encuesta-mdeia-administracion.xlsx
+++ b/plantillas/encuestas/plantilla-encuesta-mdeia-administracion.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -521,130 +521,142 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>META_SEDE</t>
+          <t>Unidades MDeIA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>¿En qué sede trabajás? [meta_sede]</t>
+          <t>Departamento Administrativo Sede San Juan; Departamento Administrativo Sede San Luis; ECRyPSJ- Escuela de Cultura Religiosa y Pastoral Sede San Juan; ESEGSJ- Escuela de Seguridad Sede San Juan; FBOSCO- Facultad Don Bosco Sede Mendoza; FCEESJ- Facultad de Ciencias Económicas y Empresariales Sede San Juan; FCEESL- Facultad de Ciencias Económicas y Empresariales Sede San Luis; FCMSJ- Facultad de Ciencias Médicas Sede San Juan; FCMSL- Facultad de Ciencias Médicas Sede San Luis; FCQyTSJ- Facultad de Ciencias Químicas y Tecnológicas Sede San Juan; FCVSL- Facultad de Ciencias Veterinarias Sede San Luis; FDCSSJ- Facultad de Derecho y Ciencias Sociales Sede San Juan; FDCSSL- Facultad de Derecho y Ciencias Sociales Sede San Luis; FFyHSJ- Facultad de Filosofía y Humanidades Sede San Juan; ISB- Instituto de Formación Docente San Buenaventura Sede San Juan; ISDSM- Instituto de Formación Docente Santa María Sede San Juan; OIA- Observatorio de Inteligencia Artificial; Secretaría de Extensión; Secretaría de Investigación; UCCuyo — Universidad Católica de Cuyo (institución completa)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>META_AREA</t>
+          <t>META_SEDE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Área o departamento (ej. Depto. Administrativo SJ, Secretaría académica) [texto]</t>
+          <t>¿En qué sede trabajás? [meta_sede]</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>IND_SIU__uso_diario</t>
+          <t>META_AREA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>¿Con qué frecuencia usás SIU-Guaraní u otros sistemas de gestión académica en tu trabajo diario? [frecuencia]</t>
+          <t>Área o unidad institucional (lista oficial MDeIA UCCuyo) [meta_unidad]</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IND_SIU__satisfaccion</t>
+          <t>IND_SIU__uso_diario</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>¿Qué tan satisfecho/a estás con los sistemas de gestión académica (SIU, etc.)? [acuerdo_5]</t>
+          <t>¿Con qué frecuencia usás SIU-Guaraní u otros sistemas de gestión académica en tu trabajo diario? [frecuencia]</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>IND_CAU__contacto</t>
+          <t>IND_SIU__satisfaccion</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>¿Contactaste al CAU / mesa de ayuda TI en los últimos 12 meses? [si_no]</t>
+          <t>¿Qué tan satisfecho/a estás con los sistemas de gestión académica (SIU, etc.)? [acuerdo_5]</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>IND_CAU__resolvio</t>
+          <t>IND_CAU__contacto</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Si contactaste, ¿el problema quedó resuelto satisfactoriamente? [si_no]</t>
+          <t>¿Contactaste al CAU / mesa de ayuda TI en los últimos 12 meses? [si_no]</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>IND_CAU__satisfaccion</t>
+          <t>IND_CAU__resolvio</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>¿Qué tan satisfecho/a estás con el soporte TI recibido? [acuerdo_5]</t>
+          <t>Si contactaste, ¿el problema quedó resuelto satisfactoriamente? [si_no]</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IND_TRAMITES__digitalizados</t>
+          <t>IND_CAU__satisfaccion</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>¿En qué nivel los trámites de tu área están digitalizados y son usables sin papel? [madurez]</t>
+          <t>¿Qué tan satisfecho/a estás con el soporte TI recibido? [acuerdo_5]</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IND_CAPACITACION_DIGITAL</t>
+          <t>IND_TRAMITES__digitalizados</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>¿En qué nivel recibís capacitación en herramientas digitales para tu puesto? [madurez]</t>
+          <t>¿En qué nivel los trámites de tu área están digitalizados y son usables sin papel? [madurez]</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IND_PSERVTI__calidad</t>
+          <t>IND_CAPACITACION_DIGITAL</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>¿En qué nivel los servicios TI que usás son confiables, oportunos y adecuados a tu trabajo? [madurez]</t>
+          <t>¿En qué nivel recibís capacitación en herramientas digitales para tu puesto? [madurez]</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>IND_PSERVTI__calidad</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>¿En qué nivel los servicios TI que usás son confiables, oportunos y adecuados a tu trabajo? [madurez]</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>IND_GESTION__satisfaccion</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>¿Qué tan satisfecho/a estás con las herramientas de gestión administrativa (compras, mesa de entrada, etc.)? [acuerdo_5]</t>
         </is>

</xml_diff>